<commit_message>
Update Neoverse content: new Digital Masqs, backgrounds, Magic Triangle Classic
</commit_message>
<xml_diff>
--- a/source/spreadsheets/Neoverse_for_Claude.xlsx
+++ b/source/spreadsheets/Neoverse_for_Claude.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmestes87/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8553947-3CDE-0046-AF16-3B19052760DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6D2337-9586-9642-898E-7CCF733D0A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{BF29D5B1-F294-134E-8F7B-70D5B4D848F8}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{BF29D5B1-F294-134E-8F7B-70D5B4D848F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1 (2)" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="162">
   <si>
     <t>Neoverse Interactive Edition</t>
   </si>
@@ -498,6 +498,33 @@
   </si>
   <si>
     <t>Photo Pop</t>
+  </si>
+  <si>
+    <t>TD End Zone</t>
+  </si>
+  <si>
+    <t>TD Fourth Down</t>
+  </si>
+  <si>
+    <t>TD Game Day</t>
+  </si>
+  <si>
+    <t>HR Full Count</t>
+  </si>
+  <si>
+    <t>HR Grand Slam</t>
+  </si>
+  <si>
+    <t>HR Stolen Base</t>
+  </si>
+  <si>
+    <t>Festive Skulls</t>
+  </si>
+  <si>
+    <t>Halloween Dance</t>
+  </si>
+  <si>
+    <t>Magic Triangle Classic</t>
   </si>
 </sst>
 </file>
@@ -884,7 +911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7152A363-982E-1044-8657-DA2C0F17B383}">
-  <dimension ref="A1:I148"/>
+  <dimension ref="A1:I157"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.5" bestFit="1" customWidth="1"/>
@@ -1731,7 +1758,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>20</v>
+        <v>159</v>
       </c>
       <c r="B39" t="s">
         <v>6</v>
@@ -1749,12 +1776,12 @@
         <v>0</v>
       </c>
       <c r="I39">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B40" t="s">
         <v>6</v>
@@ -1777,7 +1804,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B41" t="s">
         <v>6</v>
@@ -1800,126 +1827,128 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>22</v>
+      </c>
+      <c r="B42" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" t="s">
+        <v>7</v>
+      </c>
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>160</v>
+      </c>
+      <c r="B43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43" t="s">
+        <v>7</v>
+      </c>
+      <c r="G43">
+        <v>1</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
         <v>23</v>
       </c>
-      <c r="B42" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" t="s">
-        <v>6</v>
-      </c>
-      <c r="D42" t="s">
-        <v>7</v>
-      </c>
-      <c r="G42">
-        <v>1</v>
-      </c>
-      <c r="H42">
-        <v>0</v>
-      </c>
-      <c r="I42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
+      <c r="B44" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44" t="s">
+        <v>7</v>
+      </c>
+      <c r="G44">
+        <v>1</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D43" s="2"/>
-      <c r="G43">
-        <v>1</v>
-      </c>
-      <c r="H43">
-        <v>0</v>
-      </c>
-      <c r="I43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A44" s="2" t="s">
+      <c r="B45" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45" s="2"/>
+      <c r="G45">
+        <v>1</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D44" s="2"/>
-      <c r="G44">
-        <v>1</v>
-      </c>
-      <c r="H44">
-        <v>0</v>
-      </c>
-      <c r="I44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="B46" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D46" s="2"/>
+      <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="H46">
+        <v>0</v>
+      </c>
+      <c r="I46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>26</v>
       </c>
-      <c r="B45" t="s">
-        <v>6</v>
-      </c>
-      <c r="C45" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" t="s">
-        <v>7</v>
-      </c>
-      <c r="G45">
-        <v>1</v>
-      </c>
-      <c r="H45">
-        <v>0</v>
-      </c>
-      <c r="I45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>27</v>
-      </c>
-      <c r="B46" t="s">
-        <v>6</v>
-      </c>
-      <c r="C46" t="s">
-        <v>6</v>
-      </c>
-      <c r="D46" t="s">
-        <v>7</v>
-      </c>
-      <c r="G46">
-        <v>1</v>
-      </c>
-      <c r="H46">
-        <v>0</v>
-      </c>
-      <c r="I46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A47" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D47" s="2"/>
+      <c r="B47" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" t="s">
+        <v>7</v>
+      </c>
       <c r="G47">
         <v>1</v>
       </c>
@@ -1932,61 +1961,61 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
+        <v>27</v>
+      </c>
+      <c r="B48" t="s">
+        <v>6</v>
+      </c>
+      <c r="C48" t="s">
+        <v>6</v>
+      </c>
+      <c r="D48" t="s">
+        <v>7</v>
+      </c>
+      <c r="G48">
+        <v>1</v>
+      </c>
+      <c r="H48">
+        <v>0</v>
+      </c>
+      <c r="I48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D49" s="2"/>
+      <c r="G49">
+        <v>1</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>29</v>
       </c>
-      <c r="B48" t="s">
-        <v>6</v>
-      </c>
-      <c r="C48" t="s">
-        <v>6</v>
-      </c>
-      <c r="D48" t="s">
-        <v>7</v>
-      </c>
-      <c r="G48">
-        <v>1</v>
-      </c>
-      <c r="H48">
-        <v>0</v>
-      </c>
-      <c r="I48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>30</v>
-      </c>
-      <c r="B49" t="s">
-        <v>6</v>
-      </c>
-      <c r="C49" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" t="s">
-        <v>7</v>
-      </c>
-      <c r="G49">
-        <v>1</v>
-      </c>
-      <c r="H49">
-        <v>0</v>
-      </c>
-      <c r="I49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D50" s="2"/>
+      <c r="B50" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" t="s">
+        <v>6</v>
+      </c>
+      <c r="D50" t="s">
+        <v>7</v>
+      </c>
       <c r="G50">
         <v>1</v>
       </c>
@@ -1999,7 +2028,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B51" t="s">
         <v>6</v>
@@ -2021,18 +2050,16 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>33</v>
-      </c>
-      <c r="B52" t="s">
-        <v>6</v>
-      </c>
-      <c r="C52" t="s">
-        <v>6</v>
-      </c>
-      <c r="D52" t="s">
-        <v>7</v>
-      </c>
+      <c r="A52" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D52" s="2"/>
       <c r="G52">
         <v>1</v>
       </c>
@@ -2045,7 +2072,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B53" t="s">
         <v>6</v>
@@ -2068,7 +2095,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B54" t="s">
         <v>6</v>
@@ -2091,7 +2118,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B55" t="s">
         <v>6</v>
@@ -2113,16 +2140,18 @@
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A56" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D56" s="2"/>
+      <c r="A56" t="s">
+        <v>35</v>
+      </c>
+      <c r="B56" t="s">
+        <v>6</v>
+      </c>
+      <c r="C56" t="s">
+        <v>6</v>
+      </c>
+      <c r="D56" t="s">
+        <v>7</v>
+      </c>
       <c r="G56">
         <v>1</v>
       </c>
@@ -2135,7 +2164,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B57" t="s">
         <v>6</v>
@@ -2157,18 +2186,16 @@
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>39</v>
-      </c>
-      <c r="B58" t="s">
-        <v>6</v>
-      </c>
-      <c r="C58" t="s">
-        <v>6</v>
-      </c>
-      <c r="D58" t="s">
-        <v>7</v>
-      </c>
+      <c r="A58" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D58" s="2"/>
       <c r="G58">
         <v>1</v>
       </c>
@@ -2181,7 +2208,7 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B59" t="s">
         <v>6</v>
@@ -2204,7 +2231,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B60" t="s">
         <v>6</v>
@@ -2227,7 +2254,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B61" t="s">
         <v>6</v>
@@ -2250,7 +2277,7 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B62" t="s">
         <v>6</v>
@@ -2273,7 +2300,7 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B63" t="s">
         <v>6</v>
@@ -2296,7 +2323,7 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B64" t="s">
         <v>6</v>
@@ -2319,7 +2346,7 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B65" t="s">
         <v>6</v>
@@ -2342,7 +2369,7 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B66" t="s">
         <v>6</v>
@@ -2365,7 +2392,7 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B67" t="s">
         <v>6</v>
@@ -2388,89 +2415,91 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
+        <v>47</v>
+      </c>
+      <c r="B68" t="s">
+        <v>6</v>
+      </c>
+      <c r="C68" t="s">
+        <v>6</v>
+      </c>
+      <c r="D68" t="s">
+        <v>7</v>
+      </c>
+      <c r="G68">
+        <v>1</v>
+      </c>
+      <c r="H68">
+        <v>0</v>
+      </c>
+      <c r="I68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B69" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" t="s">
+        <v>6</v>
+      </c>
+      <c r="D69" t="s">
+        <v>7</v>
+      </c>
+      <c r="G69">
+        <v>1</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>49</v>
       </c>
-      <c r="B68" t="s">
-        <v>6</v>
-      </c>
-      <c r="C68" t="s">
-        <v>6</v>
-      </c>
-      <c r="D68" t="s">
-        <v>7</v>
-      </c>
-      <c r="G68">
-        <v>1</v>
-      </c>
-      <c r="H68">
-        <v>0</v>
-      </c>
-      <c r="I68">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A70" s="1" t="s">
+      <c r="B70" t="s">
+        <v>6</v>
+      </c>
+      <c r="C70" t="s">
+        <v>6</v>
+      </c>
+      <c r="D70" t="s">
+        <v>7</v>
+      </c>
+      <c r="G70">
+        <v>1</v>
+      </c>
+      <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
         <v>73</v>
       </c>
-      <c r="B71" t="s">
-        <v>6</v>
-      </c>
-      <c r="C71" t="s">
-        <v>6</v>
-      </c>
-      <c r="D71" t="s">
-        <v>7</v>
-      </c>
-      <c r="G71">
-        <v>1</v>
-      </c>
-      <c r="H71">
-        <v>0</v>
-      </c>
-      <c r="I71">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>74</v>
-      </c>
-      <c r="B72" t="s">
-        <v>6</v>
-      </c>
-      <c r="C72" t="s">
-        <v>6</v>
-      </c>
-      <c r="D72" t="s">
-        <v>7</v>
-      </c>
-      <c r="G72">
-        <v>1</v>
-      </c>
-      <c r="H72">
-        <v>0</v>
-      </c>
-      <c r="I72">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A73" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D73" s="2"/>
+      <c r="B73" t="s">
+        <v>6</v>
+      </c>
+      <c r="C73" t="s">
+        <v>6</v>
+      </c>
+      <c r="D73" t="s">
+        <v>7</v>
+      </c>
       <c r="G73">
         <v>1</v>
       </c>
@@ -2483,7 +2512,7 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B74" t="s">
         <v>6</v>
@@ -2505,18 +2534,16 @@
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>77</v>
-      </c>
-      <c r="B75" t="s">
-        <v>6</v>
-      </c>
-      <c r="C75" t="s">
-        <v>6</v>
-      </c>
-      <c r="D75" t="s">
-        <v>7</v>
-      </c>
+      <c r="A75" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D75" s="2"/>
       <c r="G75">
         <v>1</v>
       </c>
@@ -2529,7 +2556,7 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B76" t="s">
         <v>6</v>
@@ -2552,7 +2579,7 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B77" t="s">
         <v>6</v>
@@ -2575,7 +2602,7 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B78" t="s">
         <v>6</v>
@@ -2597,16 +2624,18 @@
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A79" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D79" s="2"/>
+      <c r="A79" t="s">
+        <v>79</v>
+      </c>
+      <c r="B79" t="s">
+        <v>6</v>
+      </c>
+      <c r="C79" t="s">
+        <v>6</v>
+      </c>
+      <c r="D79" t="s">
+        <v>7</v>
+      </c>
       <c r="G79">
         <v>1</v>
       </c>
@@ -2619,7 +2648,7 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B80" t="s">
         <v>6</v>
@@ -2642,7 +2671,7 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>6</v>
@@ -2662,62 +2691,60 @@
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A82" s="2" t="s">
+      <c r="A82" t="s">
+        <v>82</v>
+      </c>
+      <c r="B82" t="s">
+        <v>6</v>
+      </c>
+      <c r="C82" t="s">
+        <v>6</v>
+      </c>
+      <c r="D82" t="s">
+        <v>7</v>
+      </c>
+      <c r="G82">
+        <v>1</v>
+      </c>
+      <c r="H82">
+        <v>0</v>
+      </c>
+      <c r="I82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A83" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D83" s="2"/>
+      <c r="G83">
+        <v>1</v>
+      </c>
+      <c r="H83">
+        <v>0</v>
+      </c>
+      <c r="I83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A84" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B82" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D82" s="2"/>
-      <c r="G82">
-        <v>1</v>
-      </c>
-      <c r="H82">
-        <v>0</v>
-      </c>
-      <c r="I82">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>85</v>
-      </c>
-      <c r="B83" t="s">
-        <v>6</v>
-      </c>
-      <c r="C83" t="s">
-        <v>6</v>
-      </c>
-      <c r="D83" t="s">
-        <v>7</v>
-      </c>
-      <c r="G83">
-        <v>1</v>
-      </c>
-      <c r="H83">
-        <v>0</v>
-      </c>
-      <c r="I83">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>86</v>
-      </c>
-      <c r="B84" t="s">
-        <v>6</v>
-      </c>
-      <c r="C84" t="s">
-        <v>6</v>
-      </c>
-      <c r="D84" t="s">
-        <v>7</v>
-      </c>
+      <c r="B84" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D84" s="2"/>
       <c r="G84">
         <v>1</v>
       </c>
@@ -2730,7 +2757,7 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B85" t="s">
         <v>6</v>
@@ -2753,7 +2780,7 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B86" t="s">
         <v>6</v>
@@ -2776,7 +2803,7 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B87" t="s">
         <v>6</v>
@@ -2799,7 +2826,7 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B88" t="s">
         <v>6</v>
@@ -2822,7 +2849,7 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B89" t="s">
         <v>6</v>
@@ -2844,16 +2871,18 @@
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A90" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D90" s="2"/>
+      <c r="A90" t="s">
+        <v>156</v>
+      </c>
+      <c r="B90" t="s">
+        <v>6</v>
+      </c>
+      <c r="C90" t="s">
+        <v>6</v>
+      </c>
+      <c r="D90" t="s">
+        <v>7</v>
+      </c>
       <c r="G90">
         <v>1</v>
       </c>
@@ -2861,20 +2890,22 @@
         <v>0</v>
       </c>
       <c r="I90">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A91" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B91" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D91" s="2"/>
+      <c r="A91" t="s">
+        <v>157</v>
+      </c>
+      <c r="B91" t="s">
+        <v>6</v>
+      </c>
+      <c r="C91" t="s">
+        <v>6</v>
+      </c>
+      <c r="D91" t="s">
+        <v>7</v>
+      </c>
       <c r="G91">
         <v>1</v>
       </c>
@@ -2882,12 +2913,12 @@
         <v>0</v>
       </c>
       <c r="I91">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>94</v>
+        <v>158</v>
       </c>
       <c r="B92" t="s">
         <v>6</v>
@@ -2905,12 +2936,12 @@
         <v>0</v>
       </c>
       <c r="I92">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B93" t="s">
         <v>6</v>
@@ -2932,16 +2963,18 @@
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A94" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B94" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D94" s="2"/>
+      <c r="A94" t="s">
+        <v>91</v>
+      </c>
+      <c r="B94" t="s">
+        <v>6</v>
+      </c>
+      <c r="C94" t="s">
+        <v>6</v>
+      </c>
+      <c r="D94" t="s">
+        <v>7</v>
+      </c>
       <c r="G94">
         <v>1</v>
       </c>
@@ -2953,18 +2986,16 @@
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>97</v>
-      </c>
-      <c r="B95" t="s">
-        <v>6</v>
-      </c>
-      <c r="C95" t="s">
-        <v>6</v>
-      </c>
-      <c r="D95" t="s">
-        <v>7</v>
-      </c>
+      <c r="A95" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D95" s="2"/>
       <c r="G95">
         <v>1</v>
       </c>
@@ -2977,7 +3008,7 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>6</v>
@@ -2997,16 +3028,18 @@
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A97" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D97" s="2"/>
+      <c r="A97" t="s">
+        <v>94</v>
+      </c>
+      <c r="B97" t="s">
+        <v>6</v>
+      </c>
+      <c r="C97" t="s">
+        <v>6</v>
+      </c>
+      <c r="D97" t="s">
+        <v>7</v>
+      </c>
       <c r="G97">
         <v>1</v>
       </c>
@@ -3019,7 +3052,7 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B98" t="s">
         <v>6</v>
@@ -3042,7 +3075,7 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>6</v>
@@ -3063,7 +3096,7 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>145</v>
+        <v>97</v>
       </c>
       <c r="B100" t="s">
         <v>6</v>
@@ -3081,22 +3114,20 @@
         <v>0</v>
       </c>
       <c r="I100">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
-        <v>146</v>
-      </c>
-      <c r="B101" t="s">
-        <v>6</v>
-      </c>
-      <c r="C101" t="s">
-        <v>6</v>
-      </c>
-      <c r="D101" t="s">
-        <v>7</v>
-      </c>
+      <c r="A101" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D101" s="2"/>
       <c r="G101">
         <v>1</v>
       </c>
@@ -3104,22 +3135,20 @@
         <v>0</v>
       </c>
       <c r="I101">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
-        <v>147</v>
-      </c>
-      <c r="B102" t="s">
-        <v>6</v>
-      </c>
-      <c r="C102" t="s">
-        <v>6</v>
-      </c>
-      <c r="D102" t="s">
-        <v>7</v>
-      </c>
+      <c r="A102" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D102" s="2"/>
       <c r="G102">
         <v>1</v>
       </c>
@@ -3127,12 +3156,12 @@
         <v>0</v>
       </c>
       <c r="I102">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B103" t="s">
         <v>6</v>
@@ -3154,18 +3183,16 @@
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
-        <v>103</v>
-      </c>
-      <c r="B104" t="s">
-        <v>6</v>
-      </c>
-      <c r="C104" t="s">
-        <v>6</v>
-      </c>
-      <c r="D104" t="s">
-        <v>7</v>
-      </c>
+      <c r="A104" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D104" s="2"/>
       <c r="G104">
         <v>1</v>
       </c>
@@ -3177,16 +3204,16 @@
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
-        <v>104</v>
-      </c>
-      <c r="B105" t="s">
-        <v>6</v>
-      </c>
-      <c r="C105" t="s">
-        <v>6</v>
-      </c>
-      <c r="D105" t="s">
+      <c r="A105" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D105" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G105">
@@ -3196,17 +3223,58 @@
         <v>0</v>
       </c>
       <c r="I105">
-        <v>0</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A106" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G106">
+        <v>1</v>
+      </c>
+      <c r="H106">
+        <v>0</v>
+      </c>
+      <c r="I106">
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A107" s="1" t="s">
-        <v>105</v>
+      <c r="A107" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G107">
+        <v>1</v>
+      </c>
+      <c r="H107">
+        <v>0</v>
+      </c>
+      <c r="I107">
+        <v>1</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="B108" t="s">
         <v>6</v>
@@ -3229,7 +3297,7 @@
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="B109" t="s">
         <v>6</v>
@@ -3252,7 +3320,7 @@
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="B110" t="s">
         <v>6</v>
@@ -3275,7 +3343,7 @@
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="B111" t="s">
         <v>6</v>
@@ -3298,13 +3366,13 @@
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="B112" t="s">
         <v>6</v>
       </c>
       <c r="C112" t="s">
-        <v>142</v>
+        <v>6</v>
       </c>
       <c r="D112" t="s">
         <v>7</v>
@@ -3321,7 +3389,7 @@
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="B113" t="s">
         <v>6</v>
@@ -3342,55 +3410,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
-        <v>112</v>
-      </c>
-      <c r="B114" t="s">
-        <v>6</v>
-      </c>
-      <c r="C114" t="s">
-        <v>142</v>
-      </c>
-      <c r="D114" t="s">
-        <v>7</v>
-      </c>
-      <c r="G114">
-        <v>1</v>
-      </c>
-      <c r="H114">
-        <v>0</v>
-      </c>
-      <c r="I114">
-        <v>0</v>
-      </c>
-    </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
-        <v>113</v>
-      </c>
-      <c r="B115" t="s">
-        <v>6</v>
-      </c>
-      <c r="C115" t="s">
-        <v>6</v>
-      </c>
-      <c r="D115" t="s">
-        <v>7</v>
-      </c>
-      <c r="G115">
-        <v>1</v>
-      </c>
-      <c r="H115">
-        <v>0</v>
-      </c>
-      <c r="I115">
-        <v>0</v>
+      <c r="A115" s="1" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="B116" t="s">
         <v>6</v>
@@ -3413,7 +3440,7 @@
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="B117" t="s">
         <v>6</v>
@@ -3436,7 +3463,7 @@
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>116</v>
+        <v>161</v>
       </c>
       <c r="B118" t="s">
         <v>6</v>
@@ -3454,23 +3481,64 @@
         <v>0</v>
       </c>
       <c r="I118">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>108</v>
+      </c>
+      <c r="B119" t="s">
+        <v>6</v>
+      </c>
+      <c r="C119" t="s">
+        <v>6</v>
+      </c>
+      <c r="D119" t="s">
+        <v>7</v>
+      </c>
+      <c r="G119">
+        <v>1</v>
+      </c>
+      <c r="H119">
+        <v>0</v>
+      </c>
+      <c r="I119">
         <v>0</v>
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A120" s="1" t="s">
-        <v>117</v>
+      <c r="A120" t="s">
+        <v>109</v>
+      </c>
+      <c r="B120" t="s">
+        <v>6</v>
+      </c>
+      <c r="C120" t="s">
+        <v>6</v>
+      </c>
+      <c r="D120" t="s">
+        <v>7</v>
+      </c>
+      <c r="G120">
+        <v>1</v>
+      </c>
+      <c r="H120">
+        <v>0</v>
+      </c>
+      <c r="I120">
+        <v>0</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B121" t="s">
         <v>6</v>
       </c>
       <c r="C121" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D121" t="s">
         <v>7</v>
@@ -3487,7 +3555,7 @@
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B122" t="s">
         <v>6</v>
@@ -3510,13 +3578,13 @@
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B123" t="s">
         <v>6</v>
       </c>
       <c r="C123" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D123" t="s">
         <v>7</v>
@@ -3532,16 +3600,18 @@
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A124" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D124" s="2"/>
+      <c r="A124" t="s">
+        <v>113</v>
+      </c>
+      <c r="B124" t="s">
+        <v>6</v>
+      </c>
+      <c r="C124" t="s">
+        <v>6</v>
+      </c>
+      <c r="D124" t="s">
+        <v>7</v>
+      </c>
       <c r="G124">
         <v>1</v>
       </c>
@@ -3554,7 +3624,7 @@
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B125" t="s">
         <v>6</v>
@@ -3576,16 +3646,18 @@
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A126" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="B126" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D126" s="2"/>
+      <c r="A126" t="s">
+        <v>115</v>
+      </c>
+      <c r="B126" t="s">
+        <v>6</v>
+      </c>
+      <c r="C126" t="s">
+        <v>6</v>
+      </c>
+      <c r="D126" t="s">
+        <v>7</v>
+      </c>
       <c r="G126">
         <v>1</v>
       </c>
@@ -3598,7 +3670,7 @@
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B127" t="s">
         <v>6</v>
@@ -3619,55 +3691,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A128" t="s">
-        <v>125</v>
-      </c>
-      <c r="B128" t="s">
-        <v>6</v>
-      </c>
-      <c r="C128" t="s">
-        <v>6</v>
-      </c>
-      <c r="D128" t="s">
-        <v>7</v>
-      </c>
-      <c r="G128">
-        <v>1</v>
-      </c>
-      <c r="H128">
-        <v>0</v>
-      </c>
-      <c r="I128">
-        <v>0</v>
-      </c>
-    </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A129" t="s">
-        <v>126</v>
-      </c>
-      <c r="B129" t="s">
-        <v>6</v>
-      </c>
-      <c r="C129" t="s">
-        <v>6</v>
-      </c>
-      <c r="D129" t="s">
-        <v>7</v>
-      </c>
-      <c r="G129">
-        <v>1</v>
-      </c>
-      <c r="H129">
-        <v>0</v>
-      </c>
-      <c r="I129">
-        <v>0</v>
+      <c r="A129" s="1" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="B130" t="s">
         <v>6</v>
@@ -3690,7 +3721,7 @@
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="B131" t="s">
         <v>6</v>
@@ -3713,7 +3744,7 @@
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="B132" t="s">
         <v>6</v>
@@ -3735,18 +3766,16 @@
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A133" t="s">
-        <v>130</v>
-      </c>
-      <c r="B133" t="s">
-        <v>6</v>
-      </c>
-      <c r="C133" t="s">
-        <v>6</v>
-      </c>
-      <c r="D133" t="s">
-        <v>7</v>
-      </c>
+      <c r="A133" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D133" s="2"/>
       <c r="G133">
         <v>1</v>
       </c>
@@ -3759,7 +3788,7 @@
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="B134" t="s">
         <v>6</v>
@@ -3781,18 +3810,16 @@
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A135" t="s">
-        <v>132</v>
-      </c>
-      <c r="B135" t="s">
-        <v>6</v>
-      </c>
-      <c r="C135" t="s">
-        <v>6</v>
-      </c>
-      <c r="D135" t="s">
-        <v>7</v>
-      </c>
+      <c r="A135" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D135" s="2"/>
       <c r="G135">
         <v>1</v>
       </c>
@@ -3803,29 +3830,70 @@
         <v>0</v>
       </c>
     </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A136" t="s">
+        <v>124</v>
+      </c>
+      <c r="B136" t="s">
+        <v>6</v>
+      </c>
+      <c r="C136" t="s">
+        <v>6</v>
+      </c>
+      <c r="D136" t="s">
+        <v>7</v>
+      </c>
+      <c r="G136">
+        <v>1</v>
+      </c>
+      <c r="H136">
+        <v>0</v>
+      </c>
+      <c r="I136">
+        <v>0</v>
+      </c>
+    </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A137" s="1" t="s">
-        <v>133</v>
+      <c r="A137" t="s">
+        <v>125</v>
+      </c>
+      <c r="B137" t="s">
+        <v>6</v>
+      </c>
+      <c r="C137" t="s">
+        <v>6</v>
+      </c>
+      <c r="D137" t="s">
+        <v>7</v>
+      </c>
+      <c r="G137">
+        <v>1</v>
+      </c>
+      <c r="H137">
+        <v>0</v>
+      </c>
+      <c r="I137">
+        <v>0</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="B138" t="s">
         <v>6</v>
       </c>
       <c r="C138" t="s">
-        <v>142</v>
+        <v>6</v>
       </c>
       <c r="D138" t="s">
         <v>7</v>
       </c>
       <c r="G138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H138">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I138">
         <v>0</v>
@@ -3833,64 +3901,68 @@
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="B139" t="s">
         <v>6</v>
       </c>
       <c r="C139" t="s">
-        <v>142</v>
+        <v>6</v>
       </c>
       <c r="D139" t="s">
         <v>7</v>
       </c>
       <c r="G139">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H139">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I139">
         <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A140" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B140" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C140" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D140" s="2"/>
+      <c r="A140" t="s">
+        <v>128</v>
+      </c>
+      <c r="B140" t="s">
+        <v>6</v>
+      </c>
+      <c r="C140" t="s">
+        <v>6</v>
+      </c>
+      <c r="D140" t="s">
+        <v>7</v>
+      </c>
       <c r="G140">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I140">
         <v>0</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A141" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B141" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C141" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D141" s="2"/>
+      <c r="A141" t="s">
+        <v>129</v>
+      </c>
+      <c r="B141" t="s">
+        <v>6</v>
+      </c>
+      <c r="C141" t="s">
+        <v>6</v>
+      </c>
+      <c r="D141" t="s">
+        <v>7</v>
+      </c>
       <c r="G141">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H141">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I141">
         <v>0</v>
@@ -3898,7 +3970,7 @@
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="B142" t="s">
         <v>6</v>
@@ -3910,31 +3982,33 @@
         <v>7</v>
       </c>
       <c r="G142">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I142">
         <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A143" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B143" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C143" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D143" s="2"/>
+      <c r="A143" t="s">
+        <v>131</v>
+      </c>
+      <c r="B143" t="s">
+        <v>6</v>
+      </c>
+      <c r="C143" t="s">
+        <v>6</v>
+      </c>
+      <c r="D143" t="s">
+        <v>7</v>
+      </c>
       <c r="G143">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I143">
         <v>0</v>
@@ -3942,7 +4016,7 @@
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="B144" t="s">
         <v>6</v>
@@ -3954,68 +4028,32 @@
         <v>7</v>
       </c>
       <c r="G144">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H144">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I144">
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A145" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B145" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C145" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D145" s="2"/>
-      <c r="G145">
-        <v>0</v>
-      </c>
-      <c r="H145">
-        <v>1</v>
-      </c>
-      <c r="I145">
-        <v>0</v>
-      </c>
-    </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A146" t="s">
-        <v>143</v>
-      </c>
-      <c r="B146" t="s">
-        <v>6</v>
-      </c>
-      <c r="C146" t="s">
-        <v>6</v>
-      </c>
-      <c r="D146" t="s">
-        <v>7</v>
-      </c>
-      <c r="G146">
-        <v>0</v>
-      </c>
-      <c r="H146">
-        <v>1</v>
-      </c>
-      <c r="I146">
-        <v>0</v>
+      <c r="A146" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A147" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="B147" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C147" s="2" t="s">
-        <v>6</v>
+      <c r="A147" t="s">
+        <v>134</v>
+      </c>
+      <c r="B147" t="s">
+        <v>6</v>
+      </c>
+      <c r="C147" t="s">
+        <v>142</v>
+      </c>
+      <c r="D147" t="s">
+        <v>7</v>
       </c>
       <c r="G147">
         <v>0</v>
@@ -4029,24 +4067,220 @@
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
+        <v>135</v>
+      </c>
+      <c r="B148" t="s">
+        <v>6</v>
+      </c>
+      <c r="C148" t="s">
+        <v>142</v>
+      </c>
+      <c r="D148" t="s">
+        <v>7</v>
+      </c>
+      <c r="G148">
+        <v>0</v>
+      </c>
+      <c r="H148">
+        <v>1</v>
+      </c>
+      <c r="I148">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A149" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D149" s="2"/>
+      <c r="G149">
+        <v>0</v>
+      </c>
+      <c r="H149">
+        <v>1</v>
+      </c>
+      <c r="I149">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A150" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D150" s="2"/>
+      <c r="G150">
+        <v>0</v>
+      </c>
+      <c r="H150">
+        <v>1</v>
+      </c>
+      <c r="I150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
+        <v>138</v>
+      </c>
+      <c r="B151" t="s">
+        <v>6</v>
+      </c>
+      <c r="C151" t="s">
+        <v>6</v>
+      </c>
+      <c r="D151" t="s">
+        <v>7</v>
+      </c>
+      <c r="G151">
+        <v>0</v>
+      </c>
+      <c r="H151">
+        <v>1</v>
+      </c>
+      <c r="I151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A152" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D152" s="2"/>
+      <c r="G152">
+        <v>0</v>
+      </c>
+      <c r="H152">
+        <v>1</v>
+      </c>
+      <c r="I152">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A153" t="s">
+        <v>140</v>
+      </c>
+      <c r="B153" t="s">
+        <v>6</v>
+      </c>
+      <c r="C153" t="s">
+        <v>6</v>
+      </c>
+      <c r="D153" t="s">
+        <v>7</v>
+      </c>
+      <c r="G153">
+        <v>0</v>
+      </c>
+      <c r="H153">
+        <v>1</v>
+      </c>
+      <c r="I153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A154" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D154" s="2"/>
+      <c r="G154">
+        <v>0</v>
+      </c>
+      <c r="H154">
+        <v>1</v>
+      </c>
+      <c r="I154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A155" t="s">
+        <v>143</v>
+      </c>
+      <c r="B155" t="s">
+        <v>6</v>
+      </c>
+      <c r="C155" t="s">
+        <v>6</v>
+      </c>
+      <c r="D155" t="s">
+        <v>7</v>
+      </c>
+      <c r="G155">
+        <v>0</v>
+      </c>
+      <c r="H155">
+        <v>1</v>
+      </c>
+      <c r="I155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A156" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G156">
+        <v>0</v>
+      </c>
+      <c r="H156">
+        <v>1</v>
+      </c>
+      <c r="I156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A157" t="s">
         <v>152</v>
       </c>
-      <c r="B148" t="s">
-        <v>6</v>
-      </c>
-      <c r="C148" t="s">
-        <v>6</v>
-      </c>
-      <c r="D148" t="s">
-        <v>7</v>
-      </c>
-      <c r="G148">
-        <v>0</v>
-      </c>
-      <c r="H148">
-        <v>1</v>
-      </c>
-      <c r="I148">
+      <c r="B157" t="s">
+        <v>6</v>
+      </c>
+      <c r="C157" t="s">
+        <v>6</v>
+      </c>
+      <c r="D157" t="s">
+        <v>7</v>
+      </c>
+      <c r="G157">
+        <v>0</v>
+      </c>
+      <c r="H157">
+        <v>1</v>
+      </c>
+      <c r="I157">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Neoverse content: remove HR/TD Digital Masqs, add new backgrounds
</commit_message>
<xml_diff>
--- a/source/spreadsheets/Neoverse_for_Claude.xlsx
+++ b/source/spreadsheets/Neoverse_for_Claude.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmestes87/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6D2337-9586-9642-898E-7CCF733D0A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{371E62B2-5E5D-9649-A9BE-1B62FFEF6F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{BF29D5B1-F294-134E-8F7B-70D5B4D848F8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="156">
   <si>
     <t>Neoverse Interactive Edition</t>
   </si>
@@ -498,24 +498,6 @@
   </si>
   <si>
     <t>Photo Pop</t>
-  </si>
-  <si>
-    <t>TD End Zone</t>
-  </si>
-  <si>
-    <t>TD Fourth Down</t>
-  </si>
-  <si>
-    <t>TD Game Day</t>
-  </si>
-  <si>
-    <t>HR Full Count</t>
-  </si>
-  <si>
-    <t>HR Grand Slam</t>
-  </si>
-  <si>
-    <t>HR Stolen Base</t>
   </si>
   <si>
     <t>Festive Skulls</t>
@@ -911,7 +893,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7152A363-982E-1044-8657-DA2C0F17B383}">
-  <dimension ref="A1:I157"/>
+  <dimension ref="A1:I151"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.5" bestFit="1" customWidth="1"/>
@@ -1758,7 +1740,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B39" t="s">
         <v>6</v>
@@ -1850,7 +1832,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B43" t="s">
         <v>6</v>
@@ -2872,7 +2854,7 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>156</v>
+        <v>90</v>
       </c>
       <c r="B90" t="s">
         <v>6</v>
@@ -2890,12 +2872,12 @@
         <v>0</v>
       </c>
       <c r="I90">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>157</v>
+        <v>91</v>
       </c>
       <c r="B91" t="s">
         <v>6</v>
@@ -2913,22 +2895,20 @@
         <v>0</v>
       </c>
       <c r="I91">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>158</v>
-      </c>
-      <c r="B92" t="s">
-        <v>6</v>
-      </c>
-      <c r="C92" t="s">
-        <v>6</v>
-      </c>
-      <c r="D92" t="s">
-        <v>7</v>
-      </c>
+      <c r="A92" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D92" s="2"/>
       <c r="G92">
         <v>1</v>
       </c>
@@ -2936,22 +2916,20 @@
         <v>0</v>
       </c>
       <c r="I92">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>90</v>
-      </c>
-      <c r="B93" t="s">
-        <v>6</v>
-      </c>
-      <c r="C93" t="s">
-        <v>6</v>
-      </c>
-      <c r="D93" t="s">
-        <v>7</v>
-      </c>
+      <c r="A93" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D93" s="2"/>
       <c r="G93">
         <v>1</v>
       </c>
@@ -2964,7 +2942,7 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B94" t="s">
         <v>6</v>
@@ -2986,16 +2964,18 @@
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A95" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B95" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D95" s="2"/>
+      <c r="A95" t="s">
+        <v>95</v>
+      </c>
+      <c r="B95" t="s">
+        <v>6</v>
+      </c>
+      <c r="C95" t="s">
+        <v>6</v>
+      </c>
+      <c r="D95" t="s">
+        <v>7</v>
+      </c>
       <c r="G95">
         <v>1</v>
       </c>
@@ -3008,7 +2988,7 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>6</v>
@@ -3029,7 +3009,7 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B97" t="s">
         <v>6</v>
@@ -3051,18 +3031,16 @@
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>95</v>
-      </c>
-      <c r="B98" t="s">
-        <v>6</v>
-      </c>
-      <c r="C98" t="s">
-        <v>6</v>
-      </c>
-      <c r="D98" t="s">
-        <v>7</v>
-      </c>
+      <c r="A98" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D98" s="2"/>
       <c r="G98">
         <v>1</v>
       </c>
@@ -3075,7 +3053,7 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>6</v>
@@ -3096,7 +3074,7 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B100" t="s">
         <v>6</v>
@@ -3119,7 +3097,7 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>6</v>
@@ -3139,16 +3117,18 @@
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A102" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B102" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D102" s="2"/>
+      <c r="A102" t="s">
+        <v>145</v>
+      </c>
+      <c r="B102" t="s">
+        <v>6</v>
+      </c>
+      <c r="C102" t="s">
+        <v>6</v>
+      </c>
+      <c r="D102" t="s">
+        <v>7</v>
+      </c>
       <c r="G102">
         <v>1</v>
       </c>
@@ -3161,7 +3141,7 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>100</v>
+        <v>146</v>
       </c>
       <c r="B103" t="s">
         <v>6</v>
@@ -3183,16 +3163,18 @@
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A104" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B104" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C104" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D104" s="2"/>
+      <c r="A104" t="s">
+        <v>147</v>
+      </c>
+      <c r="B104" t="s">
+        <v>6</v>
+      </c>
+      <c r="C104" t="s">
+        <v>6</v>
+      </c>
+      <c r="D104" t="s">
+        <v>7</v>
+      </c>
       <c r="G104">
         <v>1</v>
       </c>
@@ -3204,16 +3186,16 @@
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A105" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B105" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C105" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D105" s="2" t="s">
+      <c r="A105" t="s">
+        <v>102</v>
+      </c>
+      <c r="B105" t="s">
+        <v>6</v>
+      </c>
+      <c r="C105" t="s">
+        <v>6</v>
+      </c>
+      <c r="D105" t="s">
         <v>7</v>
       </c>
       <c r="G105">
@@ -3223,20 +3205,20 @@
         <v>0</v>
       </c>
       <c r="I105">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A106" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B106" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D106" s="2" t="s">
+      <c r="A106" t="s">
+        <v>103</v>
+      </c>
+      <c r="B106" t="s">
+        <v>6</v>
+      </c>
+      <c r="C106" t="s">
+        <v>6</v>
+      </c>
+      <c r="D106" t="s">
         <v>7</v>
       </c>
       <c r="G106">
@@ -3246,20 +3228,20 @@
         <v>0</v>
       </c>
       <c r="I106">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A107" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D107" s="2" t="s">
+      <c r="A107" t="s">
+        <v>104</v>
+      </c>
+      <c r="B107" t="s">
+        <v>6</v>
+      </c>
+      <c r="C107" t="s">
+        <v>6</v>
+      </c>
+      <c r="D107" t="s">
         <v>7</v>
       </c>
       <c r="G107">
@@ -3269,58 +3251,17 @@
         <v>0</v>
       </c>
       <c r="I107">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
-        <v>145</v>
-      </c>
-      <c r="B108" t="s">
-        <v>6</v>
-      </c>
-      <c r="C108" t="s">
-        <v>6</v>
-      </c>
-      <c r="D108" t="s">
-        <v>7</v>
-      </c>
-      <c r="G108">
-        <v>1</v>
-      </c>
-      <c r="H108">
-        <v>0</v>
-      </c>
-      <c r="I108">
         <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
-        <v>146</v>
-      </c>
-      <c r="B109" t="s">
-        <v>6</v>
-      </c>
-      <c r="C109" t="s">
-        <v>6</v>
-      </c>
-      <c r="D109" t="s">
-        <v>7</v>
-      </c>
-      <c r="G109">
-        <v>1</v>
-      </c>
-      <c r="H109">
-        <v>0</v>
-      </c>
-      <c r="I109">
-        <v>0</v>
+      <c r="A109" s="1" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>147</v>
+        <v>106</v>
       </c>
       <c r="B110" t="s">
         <v>6</v>
@@ -3343,7 +3284,7 @@
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B111" t="s">
         <v>6</v>
@@ -3366,7 +3307,7 @@
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>103</v>
+        <v>155</v>
       </c>
       <c r="B112" t="s">
         <v>6</v>
@@ -3384,12 +3325,12 @@
         <v>0</v>
       </c>
       <c r="I112">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B113" t="s">
         <v>6</v>
@@ -3410,14 +3351,55 @@
         <v>0</v>
       </c>
     </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>109</v>
+      </c>
+      <c r="B114" t="s">
+        <v>6</v>
+      </c>
+      <c r="C114" t="s">
+        <v>6</v>
+      </c>
+      <c r="D114" t="s">
+        <v>7</v>
+      </c>
+      <c r="G114">
+        <v>1</v>
+      </c>
+      <c r="H114">
+        <v>0</v>
+      </c>
+      <c r="I114">
+        <v>0</v>
+      </c>
+    </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A115" s="1" t="s">
-        <v>105</v>
+      <c r="A115" t="s">
+        <v>110</v>
+      </c>
+      <c r="B115" t="s">
+        <v>6</v>
+      </c>
+      <c r="C115" t="s">
+        <v>142</v>
+      </c>
+      <c r="D115" t="s">
+        <v>7</v>
+      </c>
+      <c r="G115">
+        <v>1</v>
+      </c>
+      <c r="H115">
+        <v>0</v>
+      </c>
+      <c r="I115">
+        <v>0</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B116" t="s">
         <v>6</v>
@@ -3440,13 +3422,13 @@
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B117" t="s">
         <v>6</v>
       </c>
       <c r="C117" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D117" t="s">
         <v>7</v>
@@ -3463,7 +3445,7 @@
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>161</v>
+        <v>113</v>
       </c>
       <c r="B118" t="s">
         <v>6</v>
@@ -3481,12 +3463,12 @@
         <v>0</v>
       </c>
       <c r="I118">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B119" t="s">
         <v>6</v>
@@ -3509,7 +3491,7 @@
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B120" t="s">
         <v>6</v>
@@ -3532,13 +3514,13 @@
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B121" t="s">
         <v>6</v>
       </c>
       <c r="C121" t="s">
-        <v>142</v>
+        <v>6</v>
       </c>
       <c r="D121" t="s">
         <v>7</v>
@@ -3553,55 +3535,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A122" t="s">
-        <v>111</v>
-      </c>
-      <c r="B122" t="s">
-        <v>6</v>
-      </c>
-      <c r="C122" t="s">
-        <v>6</v>
-      </c>
-      <c r="D122" t="s">
-        <v>7</v>
-      </c>
-      <c r="G122">
-        <v>1</v>
-      </c>
-      <c r="H122">
-        <v>0</v>
-      </c>
-      <c r="I122">
-        <v>0</v>
-      </c>
-    </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A123" t="s">
-        <v>112</v>
-      </c>
-      <c r="B123" t="s">
-        <v>6</v>
-      </c>
-      <c r="C123" t="s">
-        <v>142</v>
-      </c>
-      <c r="D123" t="s">
-        <v>7</v>
-      </c>
-      <c r="G123">
-        <v>1</v>
-      </c>
-      <c r="H123">
-        <v>0</v>
-      </c>
-      <c r="I123">
-        <v>0</v>
+      <c r="A123" s="1" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B124" t="s">
         <v>6</v>
@@ -3624,7 +3565,7 @@
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B125" t="s">
         <v>6</v>
@@ -3647,7 +3588,7 @@
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B126" t="s">
         <v>6</v>
@@ -3669,18 +3610,16 @@
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
-        <v>116</v>
-      </c>
-      <c r="B127" t="s">
-        <v>6</v>
-      </c>
-      <c r="C127" t="s">
-        <v>6</v>
-      </c>
-      <c r="D127" t="s">
-        <v>7</v>
-      </c>
+      <c r="A127" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D127" s="2"/>
       <c r="G127">
         <v>1</v>
       </c>
@@ -3691,14 +3630,53 @@
         <v>0</v>
       </c>
     </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>122</v>
+      </c>
+      <c r="B128" t="s">
+        <v>6</v>
+      </c>
+      <c r="C128" t="s">
+        <v>6</v>
+      </c>
+      <c r="D128" t="s">
+        <v>7</v>
+      </c>
+      <c r="G128">
+        <v>1</v>
+      </c>
+      <c r="H128">
+        <v>0</v>
+      </c>
+      <c r="I128">
+        <v>0</v>
+      </c>
+    </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A129" s="1" t="s">
-        <v>117</v>
+      <c r="A129" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D129" s="2"/>
+      <c r="G129">
+        <v>1</v>
+      </c>
+      <c r="H129">
+        <v>0</v>
+      </c>
+      <c r="I129">
+        <v>0</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B130" t="s">
         <v>6</v>
@@ -3721,7 +3699,7 @@
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B131" t="s">
         <v>6</v>
@@ -3744,7 +3722,7 @@
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B132" t="s">
         <v>6</v>
@@ -3766,16 +3744,18 @@
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A133" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="B133" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C133" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D133" s="2"/>
+      <c r="A133" t="s">
+        <v>127</v>
+      </c>
+      <c r="B133" t="s">
+        <v>6</v>
+      </c>
+      <c r="C133" t="s">
+        <v>6</v>
+      </c>
+      <c r="D133" t="s">
+        <v>7</v>
+      </c>
       <c r="G133">
         <v>1</v>
       </c>
@@ -3788,7 +3768,7 @@
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B134" t="s">
         <v>6</v>
@@ -3810,16 +3790,18 @@
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A135" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="B135" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C135" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D135" s="2"/>
+      <c r="A135" t="s">
+        <v>129</v>
+      </c>
+      <c r="B135" t="s">
+        <v>6</v>
+      </c>
+      <c r="C135" t="s">
+        <v>6</v>
+      </c>
+      <c r="D135" t="s">
+        <v>7</v>
+      </c>
       <c r="G135">
         <v>1</v>
       </c>
@@ -3832,7 +3814,7 @@
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B136" t="s">
         <v>6</v>
@@ -3855,7 +3837,7 @@
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B137" t="s">
         <v>6</v>
@@ -3878,7 +3860,7 @@
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B138" t="s">
         <v>6</v>
@@ -3899,70 +3881,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A139" t="s">
-        <v>127</v>
-      </c>
-      <c r="B139" t="s">
-        <v>6</v>
-      </c>
-      <c r="C139" t="s">
-        <v>6</v>
-      </c>
-      <c r="D139" t="s">
-        <v>7</v>
-      </c>
-      <c r="G139">
-        <v>1</v>
-      </c>
-      <c r="H139">
-        <v>0</v>
-      </c>
-      <c r="I139">
-        <v>0</v>
-      </c>
-    </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A140" t="s">
-        <v>128</v>
-      </c>
-      <c r="B140" t="s">
-        <v>6</v>
-      </c>
-      <c r="C140" t="s">
-        <v>6</v>
-      </c>
-      <c r="D140" t="s">
-        <v>7</v>
-      </c>
-      <c r="G140">
-        <v>1</v>
-      </c>
-      <c r="H140">
-        <v>0</v>
-      </c>
-      <c r="I140">
-        <v>0</v>
+      <c r="A140" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B141" t="s">
         <v>6</v>
       </c>
       <c r="C141" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D141" t="s">
         <v>7</v>
       </c>
       <c r="G141">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H141">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I141">
         <v>0</v>
@@ -3970,87 +3911,122 @@
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B142" t="s">
         <v>6</v>
       </c>
       <c r="C142" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D142" t="s">
         <v>7</v>
       </c>
       <c r="G142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H142">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I142">
         <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A143" t="s">
-        <v>131</v>
-      </c>
-      <c r="B143" t="s">
-        <v>6</v>
-      </c>
-      <c r="C143" t="s">
-        <v>6</v>
-      </c>
-      <c r="D143" t="s">
-        <v>7</v>
-      </c>
+      <c r="A143" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D143" s="2"/>
       <c r="G143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H143">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I143">
         <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A144" t="s">
-        <v>132</v>
-      </c>
-      <c r="B144" t="s">
-        <v>6</v>
-      </c>
-      <c r="C144" t="s">
-        <v>6</v>
-      </c>
-      <c r="D144" t="s">
-        <v>7</v>
-      </c>
+      <c r="A144" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D144" s="2"/>
       <c r="G144">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H144">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I144">
         <v>0</v>
       </c>
     </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
+        <v>138</v>
+      </c>
+      <c r="B145" t="s">
+        <v>6</v>
+      </c>
+      <c r="C145" t="s">
+        <v>6</v>
+      </c>
+      <c r="D145" t="s">
+        <v>7</v>
+      </c>
+      <c r="G145">
+        <v>0</v>
+      </c>
+      <c r="H145">
+        <v>1</v>
+      </c>
+      <c r="I145">
+        <v>0</v>
+      </c>
+    </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A146" s="1" t="s">
-        <v>133</v>
+      <c r="A146" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D146" s="2"/>
+      <c r="G146">
+        <v>0</v>
+      </c>
+      <c r="H146">
+        <v>1</v>
+      </c>
+      <c r="I146">
+        <v>0</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B147" t="s">
         <v>6</v>
       </c>
       <c r="C147" t="s">
-        <v>142</v>
+        <v>6</v>
       </c>
       <c r="D147" t="s">
         <v>7</v>
@@ -4066,18 +4042,16 @@
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A148" t="s">
-        <v>135</v>
-      </c>
-      <c r="B148" t="s">
-        <v>6</v>
-      </c>
-      <c r="C148" t="s">
-        <v>142</v>
-      </c>
-      <c r="D148" t="s">
-        <v>7</v>
-      </c>
+      <c r="A148" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D148" s="2"/>
       <c r="G148">
         <v>0</v>
       </c>
@@ -4089,16 +4063,18 @@
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A149" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C149" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D149" s="2"/>
+      <c r="A149" t="s">
+        <v>143</v>
+      </c>
+      <c r="B149" t="s">
+        <v>6</v>
+      </c>
+      <c r="C149" t="s">
+        <v>6</v>
+      </c>
+      <c r="D149" t="s">
+        <v>7</v>
+      </c>
       <c r="G149">
         <v>0</v>
       </c>
@@ -4111,15 +4087,14 @@
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A150" s="2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D150" s="2"/>
+        <v>6</v>
+      </c>
       <c r="G150">
         <v>0</v>
       </c>
@@ -4132,7 +4107,7 @@
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="B151" t="s">
         <v>6</v>
@@ -4150,137 +4125,6 @@
         <v>1</v>
       </c>
       <c r="I151">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A152" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B152" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C152" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D152" s="2"/>
-      <c r="G152">
-        <v>0</v>
-      </c>
-      <c r="H152">
-        <v>1</v>
-      </c>
-      <c r="I152">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A153" t="s">
-        <v>140</v>
-      </c>
-      <c r="B153" t="s">
-        <v>6</v>
-      </c>
-      <c r="C153" t="s">
-        <v>6</v>
-      </c>
-      <c r="D153" t="s">
-        <v>7</v>
-      </c>
-      <c r="G153">
-        <v>0</v>
-      </c>
-      <c r="H153">
-        <v>1</v>
-      </c>
-      <c r="I153">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A154" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B154" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D154" s="2"/>
-      <c r="G154">
-        <v>0</v>
-      </c>
-      <c r="H154">
-        <v>1</v>
-      </c>
-      <c r="I154">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A155" t="s">
-        <v>143</v>
-      </c>
-      <c r="B155" t="s">
-        <v>6</v>
-      </c>
-      <c r="C155" t="s">
-        <v>6</v>
-      </c>
-      <c r="D155" t="s">
-        <v>7</v>
-      </c>
-      <c r="G155">
-        <v>0</v>
-      </c>
-      <c r="H155">
-        <v>1</v>
-      </c>
-      <c r="I155">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A156" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="B156" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C156" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G156">
-        <v>0</v>
-      </c>
-      <c r="H156">
-        <v>1</v>
-      </c>
-      <c r="I156">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A157" t="s">
-        <v>152</v>
-      </c>
-      <c r="B157" t="s">
-        <v>6</v>
-      </c>
-      <c r="C157" t="s">
-        <v>6</v>
-      </c>
-      <c r="D157" t="s">
-        <v>7</v>
-      </c>
-      <c r="G157">
-        <v>0</v>
-      </c>
-      <c r="H157">
-        <v>1</v>
-      </c>
-      <c r="I157">
         <v>1</v>
       </c>
     </row>

</xml_diff>